<commit_message>
nuove cartoline e sticker
</commit_message>
<xml_diff>
--- a/cartoline.xlsx
+++ b/cartoline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raffaelebalzano/Documents/Pausilypon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E001AC8-4639-7441-8E31-8E047439F678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A4E7AD-8225-5C44-90D7-BD44681FBA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="15000" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cartoline" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="85">
   <si>
     <t>titolo</t>
   </si>
@@ -76,9 +76,6 @@
     <t>La vista su Positano alla fine del sentiero degli Dei è spettacolare</t>
   </si>
   <si>
-    <t>limone</t>
-  </si>
-  <si>
     <t>IMG_9743.JPG</t>
   </si>
   <si>
@@ -122,13 +119,169 @@
   </si>
   <si>
     <t>IMG_2162.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9684.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9685.JPG</t>
+  </si>
+  <si>
+    <t>Il Faro</t>
+  </si>
+  <si>
+    <t>IMG_9690.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9686.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9687.JPG</t>
+  </si>
+  <si>
+    <t>Tuffo a mare</t>
+  </si>
+  <si>
+    <t>IMG_9694.JPG</t>
+  </si>
+  <si>
+    <t>Gioventù</t>
+  </si>
+  <si>
+    <t>IMG_9691.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9696.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9699.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9701.JPG</t>
+  </si>
+  <si>
+    <t>Partenope</t>
+  </si>
+  <si>
+    <t>IMG_9704.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9707.JPG</t>
+  </si>
+  <si>
+    <t>Tramonto su Ischia</t>
+  </si>
+  <si>
+    <t>IMG_9710.JPG</t>
+  </si>
+  <si>
+    <t>vesuvio</t>
+  </si>
+  <si>
+    <t>Turisti in viaggio</t>
+  </si>
+  <si>
+    <t>IMG_9711.JPG</t>
+  </si>
+  <si>
+    <t>Il traghetto nel golfo</t>
+  </si>
+  <si>
+    <t>IMG_9692.JPG</t>
+  </si>
+  <si>
+    <t>Maya!</t>
+  </si>
+  <si>
+    <t>IMG_9693.JPG</t>
+  </si>
+  <si>
+    <t>Il covo di Tato</t>
+  </si>
+  <si>
+    <t>IMG_9713.JPG</t>
+  </si>
+  <si>
+    <t>La terrazza di Surrient</t>
+  </si>
+  <si>
+    <t>Sorrento</t>
+  </si>
+  <si>
+    <t>limoni</t>
+  </si>
+  <si>
+    <t>IMG_9714.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9715.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9718.JPG</t>
+  </si>
+  <si>
+    <t>La piscina della Regina</t>
+  </si>
+  <si>
+    <t>Bagni Regina Giovanna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorrento </t>
+  </si>
+  <si>
+    <t>IMG_9721.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9723.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9725.JPG</t>
+  </si>
+  <si>
+    <t>Sugli scogli</t>
+  </si>
+  <si>
+    <t>IMG_9728.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9732.JPG</t>
+  </si>
+  <si>
+    <t>Checco e Dani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costiera Amalfitana </t>
+  </si>
+  <si>
+    <t>Il casolare sulla Costiera</t>
+  </si>
+  <si>
+    <t>IMG_9733.JPG</t>
+  </si>
+  <si>
+    <t>Il Sentiero degli Dei</t>
+  </si>
+  <si>
+    <t>IMG_9735.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9736.JPG</t>
+  </si>
+  <si>
+    <t>Vista sul Sentiero</t>
+  </si>
+  <si>
+    <t>IMG_9739.JPG</t>
+  </si>
+  <si>
+    <t>IMG_9741.JPG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
@@ -147,6 +300,11 @@
     <font>
       <sz val="12"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -522,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
@@ -588,7 +746,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>8</v>
@@ -597,82 +755,644 @@
         <v>17</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>33</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B25" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B27" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B33" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B36" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
napoli e suddivisione per mesi
</commit_message>
<xml_diff>
--- a/cartoline.xlsx
+++ b/cartoline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raffaelebalzano/Documents/Pausilypon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F807FF9E-5768-844A-BDE4-CA7E3D45BC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFBEA72-F29A-1E4E-9E13-84C661031942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="286">
   <si>
     <t>titolo</t>
   </si>
@@ -584,6 +584,300 @@
   </si>
   <si>
     <t>ottobre 2025</t>
+  </si>
+  <si>
+    <t>sirena</t>
+  </si>
+  <si>
+    <t>IMG_5830.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5833.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5838.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5844.JPG</t>
+  </si>
+  <si>
+    <t>Natale e Maradona</t>
+  </si>
+  <si>
+    <t>dicembre 2025</t>
+  </si>
+  <si>
+    <t>IMG_5848.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5852.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5863.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5868.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5869.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5873.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5882.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5883.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5893.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5896.JPG</t>
+  </si>
+  <si>
+    <t>Università della Strada</t>
+  </si>
+  <si>
+    <t>IMG_5898.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5901.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5903.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5905.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5906.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5907.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5912.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5914.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5918.JPG</t>
+  </si>
+  <si>
+    <t>Stai mman all'arte</t>
+  </si>
+  <si>
+    <t>IMG_5920.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5921.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5928.JPG</t>
+  </si>
+  <si>
+    <t>Sacro e Profano</t>
+  </si>
+  <si>
+    <t>IMG_5932.JPG</t>
+  </si>
+  <si>
+    <t>San Gennà</t>
+  </si>
+  <si>
+    <t>IMG_5939.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5943.JPG</t>
+  </si>
+  <si>
+    <t>Arte Presepiale</t>
+  </si>
+  <si>
+    <t>IMG_5945.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5947.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5948.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5953.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5957.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5959.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5960.JPG</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>IMG_5963.JPG</t>
+  </si>
+  <si>
+    <t>Muri puliti, Popoli muti</t>
+  </si>
+  <si>
+    <t>IMG_5964.JPG</t>
+  </si>
+  <si>
+    <t>Libri scolastici</t>
+  </si>
+  <si>
+    <t>IMG_5965.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5969.JPG</t>
+  </si>
+  <si>
+    <t>Quartieri Spagnoli</t>
+  </si>
+  <si>
+    <t>IMG_5970.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5972.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5978.JPG</t>
+  </si>
+  <si>
+    <t>IMG_5990.JPG</t>
+  </si>
+  <si>
+    <t>D10S</t>
+  </si>
+  <si>
+    <t>IMG_6000.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6009.JPG</t>
+  </si>
+  <si>
+    <t>Napulitan'</t>
+  </si>
+  <si>
+    <t>IMG_6013.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6017.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6018.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6022.JPG</t>
+  </si>
+  <si>
+    <t>Panni stesi</t>
+  </si>
+  <si>
+    <t>IMG_6025.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6032.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6035.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6044.JPG</t>
+  </si>
+  <si>
+    <t>Bene Assaje</t>
+  </si>
+  <si>
+    <t>IMG_6045.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6049.JPG</t>
+  </si>
+  <si>
+    <t>Elemosina</t>
+  </si>
+  <si>
+    <t>IMG_6050.JPG</t>
+  </si>
+  <si>
+    <t>o' cafè</t>
+  </si>
+  <si>
+    <t>IMG_6076.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6078.JPG</t>
+  </si>
+  <si>
+    <t>Plebiscito</t>
+  </si>
+  <si>
+    <t>IMG_6079.JPG</t>
+  </si>
+  <si>
+    <t>Pulcinella</t>
+  </si>
+  <si>
+    <t>IMG_6086.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6089.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6095.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6088.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6102.JPG</t>
+  </si>
+  <si>
+    <t>Dopo-scuola</t>
+  </si>
+  <si>
+    <t>081</t>
+  </si>
+  <si>
+    <t>IMG_6109.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6117.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6126.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6150.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6153.JPG</t>
+  </si>
+  <si>
+    <t>o' scalon'</t>
+  </si>
+  <si>
+    <t>o' castell' ngopp o' mar</t>
+  </si>
+  <si>
+    <t>IMG_6158.JPG</t>
+  </si>
+  <si>
+    <t>IMG_6162.JPG</t>
+  </si>
+  <si>
+    <t>Toledo sotto il mare</t>
+  </si>
+  <si>
+    <t>Napoli</t>
   </si>
 </sst>
 </file>
@@ -989,7 +1283,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G179"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
@@ -2652,7 +2946,7 @@
         <v>187</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>164</v>
@@ -2669,7 +2963,7 @@
         <v>187</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>165</v>
@@ -2686,7 +2980,7 @@
         <v>187</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>166</v>
@@ -2703,7 +2997,7 @@
         <v>187</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>167</v>
@@ -2720,7 +3014,7 @@
         <v>187</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>168</v>
@@ -2737,7 +3031,7 @@
         <v>187</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>169</v>
@@ -2754,7 +3048,7 @@
         <v>187</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>170</v>
@@ -2771,7 +3065,7 @@
         <v>187</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>171</v>
@@ -2788,7 +3082,7 @@
         <v>187</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>172</v>
@@ -2805,7 +3099,7 @@
         <v>187</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G98" s="2" t="s">
         <v>173</v>
@@ -2825,7 +3119,7 @@
         <v>187</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G99" s="2" t="s">
         <v>174</v>
@@ -2842,7 +3136,7 @@
         <v>187</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G100" s="2" t="s">
         <v>175</v>
@@ -2859,7 +3153,7 @@
         <v>187</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G101" s="2" t="s">
         <v>179</v>
@@ -2876,7 +3170,7 @@
         <v>187</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G102" s="2" t="s">
         <v>180</v>
@@ -2893,7 +3187,7 @@
         <v>187</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G103" s="2" t="s">
         <v>181</v>
@@ -2910,7 +3204,7 @@
         <v>187</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G104" s="2" t="s">
         <v>182</v>
@@ -2930,7 +3224,7 @@
         <v>187</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G105" s="2" t="s">
         <v>183</v>
@@ -2947,7 +3241,7 @@
         <v>187</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G106" s="2" t="s">
         <v>185</v>
@@ -2964,10 +3258,1304 @@
         <v>187</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>62</v>
+        <v>188</v>
       </c>
       <c r="G107" s="2" t="s">
         <v>186</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B108" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F108" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B109" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F110" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B111" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B112" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B113" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B114" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B115" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D115" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B116" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B117" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F117" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B118" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B119" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B120" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A121" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B122" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B123" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B124" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D124" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B125" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D125" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F125" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B126" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B127" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D127" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B128" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B129" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D129" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F129" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A130" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D130" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B131" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D131" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F131" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B132" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F132" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A133" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D133" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F133" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A134" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B135" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A136" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B137" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B138" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B139" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B140" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D140" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B141" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D141" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B142" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A143" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D143" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F143" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A144" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D144" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A145" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D145" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F145" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G145" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B146" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D146" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G146" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A147" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D147" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B148" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D148" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B149" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D149" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B150" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D150" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A151" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D151" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B152" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D152" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A153" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C153" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D153" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B154" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D154" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B155" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C155" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D155" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G155" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B156" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D156" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A157" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C157" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D157" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B158" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D158" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G158" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B159" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C159" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D159" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F159" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B160" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C160" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D160" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G160" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A161" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C161" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D161" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F161" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B162" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C162" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D162" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A163" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C163" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D163" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A164" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D164" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B165" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C165" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D165" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F165" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A166" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A167" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D167" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B168" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D168" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G168" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B169" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C169" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D169" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F169" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A170" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C170" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D170" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F170" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G170" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B171" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C171" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D171" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F171" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G171" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A172" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C172" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D172" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F172" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G172" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B173" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C173" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D173" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F173" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A174" s="4"/>
+      <c r="B174" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C174" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D174" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F174" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G174" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A175" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C175" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D175" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F175" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G175" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B176" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C176" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D176" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F176" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A177" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C177" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D177" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F177" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G177" s="2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B178" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C178" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D178" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F178" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G178" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A179" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C179" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="D179" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F179" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G179" s="2" t="s">
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lista raggruppata per luogo e data, con strisce di foto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cartoline.xlsx
+++ b/cartoline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raffaelebalzano/Documents/Pausilypon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47C8AF2-F7BC-D144-B4E5-FAFD2F7A3B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E931B75B-C941-1D46-9AE9-D297AE62B05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="14680" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cartoline" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1346" uniqueCount="376">
   <si>
     <t>titolo</t>
   </si>
@@ -1553,7 +1553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G253"/>
+  <dimension ref="A1:G252"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
@@ -5038,7 +5038,7 @@
         <v>373</v>
       </c>
       <c r="G191" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.2">
@@ -5055,7 +5055,7 @@
         <v>373</v>
       </c>
       <c r="G192" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="193" spans="2:7" x14ac:dyDescent="0.2">
@@ -5072,7 +5072,7 @@
         <v>373</v>
       </c>
       <c r="G193" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="194" spans="2:7" x14ac:dyDescent="0.2">
@@ -5089,7 +5089,7 @@
         <v>373</v>
       </c>
       <c r="G194" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="195" spans="2:7" x14ac:dyDescent="0.2">
@@ -5106,7 +5106,7 @@
         <v>373</v>
       </c>
       <c r="G195" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="196" spans="2:7" x14ac:dyDescent="0.2">
@@ -5123,7 +5123,7 @@
         <v>373</v>
       </c>
       <c r="G196" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="197" spans="2:7" x14ac:dyDescent="0.2">
@@ -5140,7 +5140,7 @@
         <v>373</v>
       </c>
       <c r="G197" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="198" spans="2:7" x14ac:dyDescent="0.2">
@@ -5157,7 +5157,7 @@
         <v>373</v>
       </c>
       <c r="G198" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="199" spans="2:7" x14ac:dyDescent="0.2">
@@ -5174,7 +5174,7 @@
         <v>373</v>
       </c>
       <c r="G199" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="200" spans="2:7" x14ac:dyDescent="0.2">
@@ -5191,7 +5191,7 @@
         <v>373</v>
       </c>
       <c r="G200" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="201" spans="2:7" x14ac:dyDescent="0.2">
@@ -5208,7 +5208,7 @@
         <v>373</v>
       </c>
       <c r="G201" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="202" spans="2:7" x14ac:dyDescent="0.2">
@@ -5225,7 +5225,7 @@
         <v>373</v>
       </c>
       <c r="G202" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="203" spans="2:7" x14ac:dyDescent="0.2">
@@ -5242,7 +5242,7 @@
         <v>373</v>
       </c>
       <c r="G203" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="204" spans="2:7" x14ac:dyDescent="0.2">
@@ -5259,7 +5259,7 @@
         <v>373</v>
       </c>
       <c r="G204" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="205" spans="2:7" x14ac:dyDescent="0.2">
@@ -5276,7 +5276,7 @@
         <v>373</v>
       </c>
       <c r="G205" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="206" spans="2:7" x14ac:dyDescent="0.2">
@@ -5293,7 +5293,7 @@
         <v>373</v>
       </c>
       <c r="G206" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="207" spans="2:7" x14ac:dyDescent="0.2">
@@ -5310,7 +5310,7 @@
         <v>373</v>
       </c>
       <c r="G207" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="208" spans="2:7" x14ac:dyDescent="0.2">
@@ -5327,7 +5327,7 @@
         <v>373</v>
       </c>
       <c r="G208" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="209" spans="2:7" x14ac:dyDescent="0.2">
@@ -5344,7 +5344,7 @@
         <v>373</v>
       </c>
       <c r="G209" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="210" spans="2:7" x14ac:dyDescent="0.2">
@@ -5361,7 +5361,7 @@
         <v>373</v>
       </c>
       <c r="G210" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="211" spans="2:7" x14ac:dyDescent="0.2">
@@ -5378,7 +5378,7 @@
         <v>373</v>
       </c>
       <c r="G211" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="212" spans="2:7" x14ac:dyDescent="0.2">
@@ -5395,7 +5395,7 @@
         <v>373</v>
       </c>
       <c r="G212" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="213" spans="2:7" x14ac:dyDescent="0.2">
@@ -5412,7 +5412,7 @@
         <v>373</v>
       </c>
       <c r="G213" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="214" spans="2:7" x14ac:dyDescent="0.2">
@@ -5429,7 +5429,7 @@
         <v>373</v>
       </c>
       <c r="G214" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="215" spans="2:7" x14ac:dyDescent="0.2">
@@ -5446,7 +5446,7 @@
         <v>373</v>
       </c>
       <c r="G215" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="216" spans="2:7" x14ac:dyDescent="0.2">
@@ -5463,7 +5463,7 @@
         <v>373</v>
       </c>
       <c r="G216" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="217" spans="2:7" x14ac:dyDescent="0.2">
@@ -5480,7 +5480,7 @@
         <v>373</v>
       </c>
       <c r="G217" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="218" spans="2:7" x14ac:dyDescent="0.2">
@@ -5497,7 +5497,7 @@
         <v>373</v>
       </c>
       <c r="G218" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="219" spans="2:7" x14ac:dyDescent="0.2">
@@ -5514,7 +5514,7 @@
         <v>373</v>
       </c>
       <c r="G219" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="220" spans="2:7" x14ac:dyDescent="0.2">
@@ -5531,7 +5531,7 @@
         <v>373</v>
       </c>
       <c r="G220" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="221" spans="2:7" x14ac:dyDescent="0.2">
@@ -5548,7 +5548,7 @@
         <v>373</v>
       </c>
       <c r="G221" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="222" spans="2:7" x14ac:dyDescent="0.2">
@@ -5565,7 +5565,7 @@
         <v>373</v>
       </c>
       <c r="G222" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="223" spans="2:7" x14ac:dyDescent="0.2">
@@ -5582,7 +5582,7 @@
         <v>373</v>
       </c>
       <c r="G223" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="224" spans="2:7" x14ac:dyDescent="0.2">
@@ -5599,10 +5599,13 @@
         <v>373</v>
       </c>
       <c r="G224" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A225" s="4" t="s">
+        <v>335</v>
+      </c>
       <c r="B225" s="4" t="s">
         <v>372</v>
       </c>
@@ -5616,13 +5619,10 @@
         <v>373</v>
       </c>
       <c r="G225" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A226" s="4" t="s">
-        <v>335</v>
-      </c>
       <c r="B226" s="4" t="s">
         <v>372</v>
       </c>
@@ -5636,7 +5636,7 @@
         <v>373</v>
       </c>
       <c r="G226" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.2">
@@ -5653,7 +5653,7 @@
         <v>373</v>
       </c>
       <c r="G227" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.2">
@@ -5670,7 +5670,7 @@
         <v>373</v>
       </c>
       <c r="G228" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.2">
@@ -5687,7 +5687,7 @@
         <v>373</v>
       </c>
       <c r="G229" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.2">
@@ -5704,10 +5704,13 @@
         <v>373</v>
       </c>
       <c r="G230" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A231" s="4" t="s">
+        <v>342</v>
+      </c>
       <c r="B231" s="4" t="s">
         <v>372</v>
       </c>
@@ -5721,13 +5724,10 @@
         <v>373</v>
       </c>
       <c r="G231" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A232" s="4" t="s">
-        <v>342</v>
-      </c>
       <c r="B232" s="4" t="s">
         <v>372</v>
       </c>
@@ -5741,7 +5741,7 @@
         <v>373</v>
       </c>
       <c r="G232" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.2">
@@ -5758,10 +5758,13 @@
         <v>373</v>
       </c>
       <c r="G233" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A234" s="4" t="s">
+        <v>346</v>
+      </c>
       <c r="B234" s="4" t="s">
         <v>372</v>
       </c>
@@ -5775,13 +5778,10 @@
         <v>373</v>
       </c>
       <c r="G234" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A235" s="4" t="s">
-        <v>346</v>
-      </c>
       <c r="B235" s="4" t="s">
         <v>372</v>
       </c>
@@ -5795,10 +5795,13 @@
         <v>373</v>
       </c>
       <c r="G235" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A236" s="4" t="s">
+        <v>349</v>
+      </c>
       <c r="B236" s="4" t="s">
         <v>372</v>
       </c>
@@ -5812,13 +5815,10 @@
         <v>373</v>
       </c>
       <c r="G236" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A237" s="4" t="s">
-        <v>349</v>
-      </c>
       <c r="B237" s="4" t="s">
         <v>372</v>
       </c>
@@ -5832,7 +5832,7 @@
         <v>373</v>
       </c>
       <c r="G237" s="2" t="s">
-        <v>348</v>
+        <v>359</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.2">
@@ -5849,7 +5849,7 @@
         <v>373</v>
       </c>
       <c r="G238" s="2" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.2">
@@ -5866,7 +5866,7 @@
         <v>373</v>
       </c>
       <c r="G239" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.2">
@@ -5883,10 +5883,13 @@
         <v>373</v>
       </c>
       <c r="G240" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A241" s="4" t="s">
+        <v>354</v>
+      </c>
       <c r="B241" s="4" t="s">
         <v>372</v>
       </c>
@@ -5900,13 +5903,10 @@
         <v>373</v>
       </c>
       <c r="G241" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A242" s="4" t="s">
-        <v>354</v>
-      </c>
       <c r="B242" s="4" t="s">
         <v>372</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>373</v>
       </c>
       <c r="G242" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.2">
@@ -5937,10 +5937,13 @@
         <v>373</v>
       </c>
       <c r="G243" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A244" s="4" t="s">
+        <v>358</v>
+      </c>
       <c r="B244" s="4" t="s">
         <v>372</v>
       </c>
@@ -5954,13 +5957,10 @@
         <v>373</v>
       </c>
       <c r="G244" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A245" s="4" t="s">
-        <v>358</v>
-      </c>
       <c r="B245" s="4" t="s">
         <v>372</v>
       </c>
@@ -5974,10 +5974,13 @@
         <v>373</v>
       </c>
       <c r="G245" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A246" s="4" t="s">
+        <v>362</v>
+      </c>
       <c r="B246" s="4" t="s">
         <v>372</v>
       </c>
@@ -5991,12 +5994,12 @@
         <v>373</v>
       </c>
       <c r="G246" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A247" s="4" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B247" s="4" t="s">
         <v>372</v>
@@ -6011,12 +6014,12 @@
         <v>373</v>
       </c>
       <c r="G247" s="2" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A248" s="4" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B248" s="4" t="s">
         <v>372</v>
@@ -6031,13 +6034,10 @@
         <v>373</v>
       </c>
       <c r="G248" s="2" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A249" s="4" t="s">
-        <v>366</v>
-      </c>
       <c r="B249" s="4" t="s">
         <v>372</v>
       </c>
@@ -6051,10 +6051,13 @@
         <v>373</v>
       </c>
       <c r="G249" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A250" s="4" t="s">
+        <v>369</v>
+      </c>
       <c r="B250" s="4" t="s">
         <v>372</v>
       </c>
@@ -6068,13 +6071,10 @@
         <v>373</v>
       </c>
       <c r="G250" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A251" s="4" t="s">
-        <v>369</v>
-      </c>
       <c r="B251" s="4" t="s">
         <v>372</v>
       </c>
@@ -6088,7 +6088,7 @@
         <v>373</v>
       </c>
       <c r="G251" s="2" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.2">
@@ -6105,23 +6105,6 @@
         <v>373</v>
       </c>
       <c r="G252" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B253" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="C253" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="D253" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="F253" s="4" t="s">
-        <v>373</v>
-      </c>
-      <c r="G253" s="2" t="s">
         <v>371</v>
       </c>
     </row>

</xml_diff>